<commit_message>
Cleanup repository and sync local databases
</commit_message>
<xml_diff>
--- a/samples/sample-upload.xlsx
+++ b/samples/sample-upload.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY PROJECTS\Prog\RepricerV1DB\repricer-db\samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY PROJECTS\Prog\MarketRevisorV1.2\repricer_data\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F22C02-87D1-437F-9DB7-AFA83F0695CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3996CB-D94A-449E-A461-4F7C570CD4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="2445" windowWidth="21510" windowHeight="12600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ID</t>
   </si>
@@ -37,6 +40,12 @@
   </si>
   <si>
     <t>rejectedIds</t>
+  </si>
+  <si>
+    <t>seller</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -354,10 +363,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -369,6 +378,12 @@
       </c>
       <c r="D1" t="s">
         <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>